<commit_message>
fix(i18n): sync psychology translations, fix Echarts axis formatting and standardize Fiscal texts
</commit_message>
<xml_diff>
--- a/Profit_RTD.xlsx
+++ b/Profit_RTD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJETOS\TraderLogPro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B99398-CC98-4BCC-8634-A3009DDC6F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E15778-42B5-4253-9831-E5C420269DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1900" yWindow="1900" windowWidth="25800" windowHeight="10010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="117">
   <si>
     <t>Asset</t>
   </si>
@@ -392,9 +392,6 @@
   <si>
     <t xml:space="preserve"> </t>
   </si>
-  <si>
-    <t>psicotrade</t>
-  </si>
 </sst>
 </file>
 
@@ -3443,13 +3440,6 @@
         <stp>IMPVT</stp>
         <tr r="AN29" s="1"/>
       </tp>
-      <tp t="s">
-        <v>Atributo Inválido</v>
-        <stp/>
-        <stp>WINFUT_F_0</stp>
-        <stp>101_psicotrade</stp>
-        <tr r="AZ3" s="2"/>
-      </tp>
       <tp t="b">
         <v>0</v>
         <stp/>
@@ -3842,13 +3832,6 @@
         <stp>DOBRAR</stp>
         <tr r="AV2" s="1"/>
       </tp>
-      <tp t="s">
-        <v>Atributo Inválido</v>
-        <stp/>
-        <stp>WDOFUT_F_0</stp>
-        <stp>101_psicotrade</stp>
-        <tr r="AZ2" s="2"/>
-      </tp>
       <tp t="b">
         <v>0</v>
         <stp/>
@@ -5557,13 +5540,6 @@
         <stp>VARPTS</stp>
         <tr r="K3" s="2"/>
       </tp>
-      <tp t="s">
-        <v>Atributo Inválido</v>
-        <stp/>
-        <stp>BITFUT_F_0</stp>
-        <stp>101_psicotrade</stp>
-        <tr r="AZ4" s="2"/>
-      </tp>
       <tp t="b">
         <v>0</v>
         <stp/>
@@ -11057,6 +11033,7 @@
         <stp/>
         <stp>BITFUT_F_0</stp>
         <stp>67</stp>
+        <tr r="AZ4" s="2"/>
         <tr r="BA4" s="2"/>
       </tp>
       <tp t="b">
@@ -11589,6 +11566,7 @@
         <stp/>
         <stp>WDOFUT_F_0</stp>
         <stp>67</stp>
+        <tr r="AZ2" s="2"/>
         <tr r="BA2" s="2"/>
       </tp>
       <tp t="b">
@@ -11617,6 +11595,7 @@
         <stp/>
         <stp>WINFUT_F_0</stp>
         <stp>67</stp>
+        <tr r="AZ3" s="2"/>
         <tr r="BA3" s="2"/>
       </tp>
       <tp t="b">
@@ -18351,7 +18330,7 @@
         <v>50</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>117</v>
+        <v>51</v>
       </c>
       <c r="BA1" s="1" t="s">
         <v>51</v>
@@ -18560,9 +18539,9 @@
         <f>RTD("rtdtrading.rtdserver",, "WDOFUT_F_0", "VEXT")</f>
         <v>0</v>
       </c>
-      <c r="AZ2" s="1" t="str">
-        <f>RTD("rtdtrading.rtdserver",, "WDOFUT_F_0", "101_psicotrade")</f>
-        <v>Atributo Inválido</v>
+      <c r="AZ2" s="1">
+        <f>RTD("rtdtrading.rtdserver",, "WDOFUT_F_0", "67")</f>
+        <v>0</v>
       </c>
       <c r="BA2" s="1">
         <f>RTD("rtdtrading.rtdserver",, "WDOFUT_F_0", "67")</f>
@@ -18772,9 +18751,9 @@
         <f>RTD("rtdtrading.rtdserver",, "WINFUT_F_0", "VEXT")</f>
         <v>0</v>
       </c>
-      <c r="AZ3" s="1" t="str">
-        <f>RTD("rtdtrading.rtdserver",, "WINFUT_F_0", "101_psicotrade")</f>
-        <v>Atributo Inválido</v>
+      <c r="AZ3" s="1">
+        <f>RTD("rtdtrading.rtdserver",, "WINFUT_F_0", "67")</f>
+        <v>0</v>
       </c>
       <c r="BA3" s="1">
         <f>RTD("rtdtrading.rtdserver",, "WINFUT_F_0", "67")</f>
@@ -18984,9 +18963,9 @@
         <f>RTD("rtdtrading.rtdserver",, "BITFUT_F_0", "VEXT")</f>
         <v>0</v>
       </c>
-      <c r="AZ4" s="1" t="str">
-        <f>RTD("rtdtrading.rtdserver",, "BITFUT_F_0", "101_psicotrade")</f>
-        <v>Atributo Inválido</v>
+      <c r="AZ4" s="1">
+        <f>RTD("rtdtrading.rtdserver",, "BITFUT_F_0", "67")</f>
+        <v>0</v>
       </c>
       <c r="BA4" s="1">
         <f>RTD("rtdtrading.rtdserver",, "BITFUT_F_0", "67")</f>

</xml_diff>